<commit_message>
feat(006): fase D — PCH e CGH em conjunto (relatório em duas partes, composição e peso na potência, período pela entrada no conjunto, códigos de programação de todo o período, hidrologia sem EVT), convergência T159–T161 e referências da PCH Bandeirante e da UFV Seriemas 1
</commit_message>
<xml_diff>
--- a/relatorios_referencia/seriemas_1/perfil_estatistico_anual.xlsx
+++ b/relatorios_referencia/seriemas_1/perfil_estatistico_anual.xlsx
@@ -30,10 +30,13 @@
     <sheet name="CONF_G2_MENSAL" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="CONF_G2_DIVERGENCIAS" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="CONF_G5_MENSAL" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="CAD_FICHA" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="CAD_AUDITORIA" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="DICIONARIOS" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="FONTES" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="CONJ_TRECHOS" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="CONJ_COMPOSICAO" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="CONJ_MENSAL" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="CAD_FICHA" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="CAD_AUDITORIA" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="DICIONARIOS" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="FONTES" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -549,10 +552,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Composição do conjunto</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>O conjunto Conj. Inocência 230 kV (CJU_MS4FINO) teve 1 composição no período: de 22/08/2026 a 19/10/2026, 8 usinas (UFV), geração média do conjunto de 66,7 MWmed. Os números são do conjunto, sem divisão entre as usinas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Qualidade dos dados</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Nenhuma hora sinalizada na base horária.</t>
         </is>
@@ -4168,6 +4183,557 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>trecho</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>inicio</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fim</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>usinas</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>tipos</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>horas</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>horas_com_valor</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>energia_mwh</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>geracao_media_mw</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>geracao_maxima_mw</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>potencia_somada_mw</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>usinas_sem_potencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46314.95833333334</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1416</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1416</v>
+      </c>
+      <c r="H2" t="n">
+        <v>94480.74549999999</v>
+      </c>
+      <c r="I2" t="n">
+        <v>66.72369032485875</v>
+      </c>
+      <c r="J2" t="n">
+        <v>393.3155</v>
+      </c>
+      <c r="K2" t="n">
+        <v>400</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>trecho</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ceg</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>usina</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>entrada</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>saida</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>unidades</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>potencia_mw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052257-0.01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Seriemas 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052258-9.01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Seriemas 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052259-7.01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Seriemas 3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052260-0.01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Seriemas 4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052261-9.01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Seriemas 5</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052262-7.01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seriemas 6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052263-5.01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Seriemas 7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UFV.RS.MS.052264-3.01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Seriemas 8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>UFV</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>mes</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>trecho</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>horas_com_valor</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>geracao_media_mw</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>energia_mwh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>240</v>
+      </c>
+      <c r="D2" t="n">
+        <v>58.9367625</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14144.823</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>720</v>
+      </c>
+      <c r="D3" t="n">
+        <v>68.72983402777777</v>
+      </c>
+      <c r="E3" t="n">
+        <v>49485.4805</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>456</v>
+      </c>
+      <c r="D4" t="n">
+        <v>67.65447807017544</v>
+      </c>
+      <c r="E4" t="n">
+        <v>30850.442</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4339,7 +4905,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4444,7 +5010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5306,756 +5872,6 @@
         <v>0</v>
       </c>
       <c r="K17" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>aba</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>conjuntos_origem</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>conferencias</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sem_outra_fonte</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>calculado_no_relatorio</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CONSTATACOES</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW)); geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CONCLUSAO</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW)); geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BASE_ANUAL</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>geração</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BASE_MENSAL</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>geração</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BASE_HORA_DO_DIA</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>geração</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TRECHOS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>OMITIDOS</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>parâmetros do projeto (origem na tabela de parâmetros)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>CONF_NAO_APLICAVEIS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>parâmetros do projeto (origem na tabela de parâmetros)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PARAMETROS</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>parâmetros do projeto (origem na tabela de parâmetros); Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>PROG_RESUMO_MENSAL</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>geração</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PROG_EVENTOS_DESVIO</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>geração</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>REN_FC_ANUAL</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>REN_FC_MENSAL</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>REN_CORTE_ANUAL</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>geração estimada e marca de restrição</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>REN_CORTE_MENSAL</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>geração estimada e marca de restrição</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>REN_CORTE_RAZAO</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>geração estimada e marca de restrição</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>REN_RECURSO_FAIXAS</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>vento ou irradiância</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>REN_DESVIOS_PROGRAMACAO</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>CONF_G1_MENSAL</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>CONF_G2_MENSAL</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>CONF_G2_DIVERGENCIAS</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>CONF_G5_MENSAL</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CAD_FICHA</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW))</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>CAD_AUDITORIA</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>DICIONARIOS</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>não</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6197,6 +6013,837 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>aba</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>conjuntos_origem</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>conferencias</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sem_outra_fonte</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>calculado_no_relatorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CONSTATACOES</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW)); geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CONCLUSAO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW)); geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BASE_ANUAL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BASE_MENSAL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BASE_HORA_DO_DIA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TRECHOS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OMITIDOS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>parâmetros do projeto (origem na tabela de parâmetros)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CONF_NAO_APLICAVEIS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>parâmetros do projeto (origem na tabela de parâmetros)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PARAMETROS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>parâmetros do projeto (origem na tabela de parâmetros); Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PROG_RESUMO_MENSAL</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PROG_EVENTOS_DESVIO</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REN_FC_ANUAL</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>REN_FC_MENSAL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; parâmetros do projeto (origem na tabela de parâmetros)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REN_CORTE_ANUAL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES; soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>geração estimada e marca de restrição</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>REN_CORTE_MENSAL</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>geração estimada e marca de restrição</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>REN_CORTE_RAZAO</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>geração estimada e marca de restrição</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>REN_RECURSO_FAIXAS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>vento ou irradiância</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>REN_DESVIOS_PROGRAMACAO</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CONF_G1_MENSAL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>geração conferida entre as fontes, duas a duas e no mesmo nível (G1): 4.248 de 4.248 horas coincidentes (100,0%) em 3 pares de fontes, detalhados na aba CONF_G1_PARES</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CONF_G2_MENSAL</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CONF_G2_DIVERGENCIAS</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CONF_G5_MENSAL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>programação diária conferida com o programado do Fator de capacidade (G5): 1.104 de 1.104 horas coincidentes (100,0%), 192 horas só numa das fontes</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CONJ_TRECHOS</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CONJ_COMPOSICAO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CONJ_MENSAL</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG das usinas do conjunto CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>soma das usinas do conjunto (Restrição com detalhe) conferida com a Geração por usina do conjunto (G2): 1.105 de 1.296 horas coincidentes (85,3%), 191 divergências, listadas na aba CONF_G2_DIVERGENCIAS; 120 horas sem todas as usinas, fora da soma</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>geração</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CAD_FICHA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>potência autorizada e estado conferidos com os parâmetros do projeto: divergências (potência autorizada de 2,5 MW (projeto: 50 MW))</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CAD_AUDITORIA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DICIONARIOS</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Programação diária (conjunto de usinas, MS4FINO), obtido em 20/10/2026; Geração por usina (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Modalidade das usinas (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Composição dos conjuntos de usinas (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Capacidade de geração (CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Fator de capacidade (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026; Restrição com detalhe (constrained-off) (id ONS MSSRI1; CEG UFV.RS.MS.052257-0.01), obtido em 21/10/2026; Restrição com a razão (constrained-off) (conjunto de usinas, id ONS CJU_MS4FINO), obtido em 21/10/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6875,7 +7522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6920,7 +7567,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Composição e geração do conjunto</t>
+          <t>Conferência da geração entre fontes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6930,31 +7577,31 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>seção ainda não gerada pelo pipeline; a composição por trecho está na Fonte e cobertura dos dados</t>
+          <t>seção ainda não gerada pelo pipeline; os resultados da G1, da G2 e da G5, quando aplicáveis, estão nas legendas de fonte das seções de eólica e solar e nas abas CONF_G1, CONF_G2 e CONF_G5 da planilha</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Conferência da geração entre fontes</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>secao</t>
+          <t>regra</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>seção ainda não gerada pelo pipeline; os resultados da G1, da G2 e da G5, quando aplicáveis, estão nas legendas de fonte das seções de eólica e solar e nas abas CONF_G1, CONF_G2 e CONF_G5 da planilha</t>
+          <t>sem o Fator de capacidade no nível da usina</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6963,23 +7610,6 @@
         </is>
       </c>
       <c r="C5" t="inlineStr">
-        <is>
-          <t>sem o Fator de capacidade no nível da usina</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>regra</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
         <is>
           <t>sem a Programação diária no nível da usina</t>
         </is>

</xml_diff>